<commit_message>
Add points for aw4mhrfav7b5r7d4lc6dwz1g4_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/aw4mhrfav7b5r7d4lc6dwz1g4_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/aw4mhrfav7b5r7d4lc6dwz1g4_playerlog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG25"/>
+  <dimension ref="A1:BG33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,14 +780,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -819,7 +819,7 @@
         <v>1</v>
       </c>
       <c r="AE2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF2" t="n">
         <v>0</v>
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -850,7 +850,7 @@
         <v>0</v>
       </c>
       <c r="AR2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS2" t="n">
         <v>0</v>
@@ -862,7 +862,7 @@
         <v>0</v>
       </c>
       <c r="AV2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -951,14 +951,14 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -990,10 +990,10 @@
         <v>1</v>
       </c>
       <c r="AE3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF3" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG3" t="n">
         <v>1</v>
@@ -1004,21 +1004,21 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>0.12702678</v>
+        <v>0.48414822</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>-0.13</t>
+          <t>+0.08</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN3" t="n">
         <v>0</v>
@@ -1030,13 +1030,13 @@
         <v>0</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AR3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT3" t="n">
         <v>1</v>
@@ -1057,7 +1057,7 @@
         <v>0</v>
       </c>
       <c r="AZ3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BA3" t="n">
         <v>0</v>
@@ -1073,7 +1073,7 @@
         <v>0</v>
       </c>
       <c r="BF3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG3" t="n">
         <v>0</v>
@@ -1120,10 +1120,12 @@
           <t>9pdikqp2g2nxvfjs1nq4fmx9l</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
@@ -1134,14 +1136,14 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1149,7 +1151,7 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -1173,13 +1175,13 @@
         <v>1</v>
       </c>
       <c r="AE4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF4" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
@@ -1187,21 +1189,21 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0.03234589</v>
+        <v>-0.2054427200000001</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>-0.23</t>
+          <t>-0.61</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
@@ -1216,16 +1218,16 @@
         <v>0</v>
       </c>
       <c r="AR4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AS4" t="n">
         <v>2</v>
       </c>
       <c r="AT4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AV4" t="n">
         <v>0</v>
@@ -1317,14 +1319,14 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1332,7 +1334,7 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
@@ -1356,10 +1358,10 @@
         <v>1</v>
       </c>
       <c r="AE5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF5" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG5" t="n">
         <v>1</v>
@@ -1370,21 +1372,21 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>0.15433969</v>
+        <v>0.01393218</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.39</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN5" t="n">
         <v>0</v>
@@ -1399,19 +1401,19 @@
         <v>1</v>
       </c>
       <c r="AR5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AS5" t="n">
         <v>0</v>
       </c>
       <c r="AT5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AU5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AV5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
@@ -1500,14 +1502,14 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1515,7 +1517,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -1539,10 +1541,10 @@
         <v>1</v>
       </c>
       <c r="AE6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF6" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG6" t="n">
         <v>1</v>
@@ -1553,21 +1555,21 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0.13513121</v>
+        <v>0.21004673</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>-0.12</t>
+          <t>-0.19</t>
         </is>
       </c>
       <c r="AK6" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AL6" t="n">
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN6" t="n">
         <v>0</v>
@@ -1585,13 +1587,13 @@
         <v>2</v>
       </c>
       <c r="AS6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV6" t="n">
         <v>0</v>
@@ -1669,10 +1671,12 @@
           <t>eb1988spb5nq8i4fb8fa6hnu1</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
@@ -1683,14 +1687,18 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>56</v>
-      </c>
-      <c r="O7" t="inlineStr"/>
+        <v>88</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1698,10 +1706,16 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>56</v>
-      </c>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+        <v>70.2</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>17.8</v>
+      </c>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
@@ -1722,13 +1736,13 @@
         <v>1</v>
       </c>
       <c r="AE7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF7" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1736,21 +1750,21 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>-0.16820341</v>
+        <v>0.06051978000000002</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>-0.43</t>
+          <t>-0.34</t>
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="AN7" t="n">
         <v>0</v>
@@ -1759,7 +1773,7 @@
         <v>0</v>
       </c>
       <c r="AP7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AQ7" t="n">
         <v>0</v>
@@ -1768,13 +1782,13 @@
         <v>1</v>
       </c>
       <c r="AS7" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU7" t="n">
         <v>4</v>
-      </c>
-      <c r="AT7" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU7" t="n">
-        <v>3</v>
       </c>
       <c r="AV7" t="n">
         <v>1</v>
@@ -1805,7 +1819,7 @@
         <v>0</v>
       </c>
       <c r="BF7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG7" t="n">
         <v>0</v>
@@ -1852,10 +1866,12 @@
           <t>dckt870up1k5s5yfblij0v7ys</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -1866,14 +1882,14 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1881,7 +1897,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -1905,13 +1921,13 @@
         <v>1</v>
       </c>
       <c r="AE8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF8" t="n">
         <v>0</v>
       </c>
       <c r="AG8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
@@ -1919,7 +1935,7 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>0.23432537</v>
+        <v>0.37195504</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
@@ -1927,13 +1943,13 @@
         </is>
       </c>
       <c r="AK8" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="AN8" t="n">
         <v>0</v>
@@ -2049,14 +2065,14 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2064,7 +2080,7 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
@@ -2088,10 +2104,10 @@
         <v>1</v>
       </c>
       <c r="AE9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF9" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG9" t="n">
         <v>1</v>
@@ -2102,21 +2118,21 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>-0.21012624</v>
+        <v>-0.08992450000000003</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>-0.47</t>
+          <t>-0.49</t>
         </is>
       </c>
       <c r="AK9" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="AL9" t="n">
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN9" t="n">
         <v>0</v>
@@ -2131,16 +2147,16 @@
         <v>0</v>
       </c>
       <c r="AR9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AS9" t="n">
         <v>2</v>
       </c>
       <c r="AT9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AV9" t="n">
         <v>0</v>
@@ -2232,14 +2248,14 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -2247,7 +2263,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
@@ -2271,7 +2287,7 @@
         <v>1</v>
       </c>
       <c r="AE10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF10" t="n">
         <v>0</v>
@@ -2285,34 +2301,34 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.48857447</v>
+        <v>0.8749804400000001</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>+0.23</t>
+          <t>+0.47</t>
         </is>
       </c>
       <c r="AK10" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>95</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ10" t="n">
         <v>4</v>
       </c>
-      <c r="AL10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>56</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>2</v>
-      </c>
       <c r="AR10" t="n">
         <v>2</v>
       </c>
@@ -2329,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="AW10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX10" t="n">
         <v>0</v>
@@ -2354,7 +2370,7 @@
         <v>0</v>
       </c>
       <c r="BF10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BG10" t="n">
         <v>0</v>
@@ -2401,10 +2417,12 @@
           <t>5ilkkfbsss0bxd6ttdlqg0uz9</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>2</v>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -2415,14 +2433,14 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2430,7 +2448,7 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
@@ -2454,13 +2472,13 @@
         <v>1</v>
       </c>
       <c r="AE11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF11" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -2468,30 +2486,30 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.7835753100000001</v>
+        <v>0.94105832</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>+0.52</t>
+          <t>+0.54</t>
         </is>
       </c>
       <c r="AK11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>75</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP11" t="n">
         <v>3</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>56</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>1</v>
       </c>
       <c r="AQ11" t="n">
         <v>3</v>
@@ -2541,10 +2559,10 @@
         <v>3</v>
       </c>
       <c r="BF11" t="n">
+        <v>7</v>
+      </c>
+      <c r="BG11" t="n">
         <v>5</v>
-      </c>
-      <c r="BG11" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -2588,10 +2606,12 @@
           <t>ebpbo82i3h1lmgvx0zop6akx6</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>2</v>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -2602,14 +2622,14 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2617,7 +2637,7 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
@@ -2641,13 +2661,13 @@
         <v>1</v>
       </c>
       <c r="AE12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF12" t="n">
         <v>0</v>
       </c>
       <c r="AG12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -2655,11 +2675,11 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>1.20603926</v>
+        <v>1.46865433</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>+0.95</t>
+          <t>+1.06</t>
         </is>
       </c>
       <c r="AK12" t="n">
@@ -2669,7 +2689,7 @@
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="AN12" t="n">
         <v>1</v>
@@ -2678,13 +2698,13 @@
         <v>0</v>
       </c>
       <c r="AP12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ12" t="n">
         <v>1</v>
       </c>
       <c r="AR12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AS12" t="n">
         <v>1</v>
@@ -2693,7 +2713,7 @@
         <v>1</v>
       </c>
       <c r="AU12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV12" t="n">
         <v>0</v>
@@ -2724,7 +2744,7 @@
         <v>0</v>
       </c>
       <c r="BF12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BG12" t="n">
         <v>0</v>
@@ -2738,37 +2758,37 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>pfvmhackqyhhk02majd2tb8l</t>
+          <t>3669sbeijslw88073qlw1cbcp</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>T. Courtois</t>
+          <t>Ramy Rabia</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t xml:space="preserve"> 5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>6crmq7vzqts58wg196q48sc7p</t>
+          <t>etjattxcqbg5g8rzmt2mbst05</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -2777,30 +2797,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>70</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="Q13" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S13" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
@@ -2812,35 +2836,47 @@
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>pfvmhackqyhhk02majd2tb8l</t>
+          <t>3669sbeijslw88073qlw1cbcp</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="AD13" t="n">
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF13" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>Ramy Rabia</t>
+        </is>
+      </c>
+      <c r="AI13" t="n">
+        <v>0.11798531</v>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>-0.29</t>
+        </is>
+      </c>
+      <c r="AK13" t="n">
+        <v>19</v>
+      </c>
       <c r="AL13" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="AM13" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN13" t="n">
         <v>0</v>
@@ -2861,13 +2897,13 @@
         <v>2</v>
       </c>
       <c r="AT13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU13" t="n">
         <v>0</v>
       </c>
       <c r="AV13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AW13" t="n">
         <v>0</v>
@@ -2890,11 +2926,7 @@
       <c r="BC13" t="n">
         <v>0</v>
       </c>
-      <c r="BD13" t="inlineStr">
-        <is>
-          <t>GK</t>
-        </is>
-      </c>
+      <c r="BD13" t="inlineStr"/>
       <c r="BE13" t="n">
         <v>0</v>
       </c>
@@ -2902,7 +2934,7 @@
         <v>0</v>
       </c>
       <c r="BG13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2913,37 +2945,37 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>pfvmhackqyhhk02majd2tb8l</t>
+          <t>3669sbeijslw88073qlw1cbcp</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>T. Meunier</t>
+          <t>Hamza Abdelkarim</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 15</t>
+          <t xml:space="preserve"> 9</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>bb6glt8n0ar47cmhmj6gnfiz9</t>
+          <t>1m3kmmbxavzv5ih3t9cwal1qs</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -2952,30 +2984,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>75</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2</v>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="Q14" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
@@ -2987,47 +3023,47 @@
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>pfvmhackqyhhk02majd2tb8l</t>
+          <t>3669sbeijslw88073qlw1cbcp</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="AD14" t="n">
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>-0.2</v>
+        <v>-0</v>
       </c>
       <c r="AG14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>T. Meunier</t>
+          <t>Hamza Abdelkarim</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.42970995</v>
+        <v>-0.08811448999999999</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>+0.17</t>
+          <t>-0.49</t>
         </is>
       </c>
       <c r="AK14" t="n">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="AL14" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="AM14" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3045,13 +3081,13 @@
         <v>1</v>
       </c>
       <c r="AS14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AT14" t="n">
         <v>0</v>
       </c>
       <c r="AU14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV14" t="n">
         <v>0</v>
@@ -3096,17 +3132,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>pfvmhackqyhhk02majd2tb8l</t>
+          <t>3669sbeijslw88073qlw1cbcp</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>T. Castagne</t>
+          <t>Karim Hafez</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 21</t>
+          <t xml:space="preserve"> 15</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3116,43 +3152,45 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>7lakmodg6ith2zbfhj6m23e8l</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>88</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>p87gxg8kc9ta6iipqt5fxmtx</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>2</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="N15" t="n">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="Q15" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -3160,7 +3198,7 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
@@ -3172,47 +3210,47 @@
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>pfvmhackqyhhk02majd2tb8l</t>
+          <t>3669sbeijslw88073qlw1cbcp</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="AD15" t="n">
         <v>0</v>
       </c>
       <c r="AE15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0.2</v>
+        <v>-0</v>
       </c>
       <c r="AG15" t="n">
         <v>2</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>T. Castagne</t>
+          <t>Karim Hafez</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>0.1234887800000001</v>
+        <v>0.08486990999999999</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>-0.14</t>
+          <t>-0.32</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="AL15" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="AM15" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN15" t="n">
         <v>0</v>
@@ -3221,31 +3259,31 @@
         <v>0</v>
       </c>
       <c r="AP15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT15" t="n">
         <v>0</v>
       </c>
       <c r="AU15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AV15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW15" t="n">
         <v>0</v>
       </c>
       <c r="AX15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY15" t="n">
         <v>0</v>
@@ -3267,7 +3305,7 @@
         <v>0</v>
       </c>
       <c r="BF15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BG15" t="n">
         <v>0</v>
@@ -3281,37 +3319,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>pfvmhackqyhhk02majd2tb8l</t>
+          <t>3669sbeijslw88073qlw1cbcp</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Y. Tielemans</t>
+          <t>Ibrahim Adel</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 8</t>
+          <t xml:space="preserve"> 20</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>eo4uva2gnx08xdazfaqzyz2dx</t>
+          <t>1ylzr03ex5mu3gs6mu8jjbvca</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -3320,30 +3358,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>88</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2</v>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="Q16" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S16" t="n">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
@@ -3355,47 +3397,47 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>pfvmhackqyhhk02majd2tb8l</t>
+          <t>3669sbeijslw88073qlw1cbcp</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="AD16" t="n">
         <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF16" t="n">
-        <v>-0.05</v>
+        <v>-0</v>
       </c>
       <c r="AG16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Y. Tielemans</t>
+          <t>Ibrahim Adel</t>
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>0.31063664</v>
+        <v>0.05090435</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>+0.05</t>
+          <t>-0.35</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="AL16" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="AM16" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN16" t="n">
         <v>0</v>
@@ -3404,13 +3446,13 @@
         <v>0</v>
       </c>
       <c r="AP16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS16" t="n">
         <v>0</v>
@@ -3419,7 +3461,7 @@
         <v>0</v>
       </c>
       <c r="AU16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV16" t="n">
         <v>0</v>
@@ -3445,19 +3487,15 @@
       <c r="BC16" t="n">
         <v>0</v>
       </c>
-      <c r="BD16" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
+      <c r="BD16" t="inlineStr"/>
       <c r="BE16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BF16" t="n">
         <v>1</v>
       </c>
       <c r="BG16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -3468,12 +3506,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>pfvmhackqyhhk02majd2tb8l</t>
+          <t>3669sbeijslw88073qlw1cbcp</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>N. Ngoy</t>
+          <t>Zizo</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -3483,22 +3521,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>a5jrqzijth7e3uxl4phi83sdm</t>
+          <t>a7s4huglg11yygt1ue0u2bit</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -3507,30 +3545,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>75</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2</v>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="Q17" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="S17" t="n">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
@@ -3542,47 +3584,47 @@
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>pfvmhackqyhhk02majd2tb8l</t>
+          <t>3669sbeijslw88073qlw1cbcp</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="AD17" t="n">
         <v>0</v>
       </c>
       <c r="AE17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF17" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>N. Ngoy</t>
+          <t>Zizo</t>
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.01234494</v>
+        <v>0.17730737</v>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.23</t>
         </is>
       </c>
       <c r="AK17" t="n">
         <v>18</v>
       </c>
       <c r="AL17" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="AM17" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3597,16 +3639,16 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV17" t="n">
         <v>0</v>
@@ -3656,17 +3698,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>B. Mechele</t>
+          <t>T. Courtois</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3676,12 +3718,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>l6y4o9t2b0jxaxo85oztok45</t>
+          <t>6crmq7vzqts58wg196q48sc7p</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -3698,22 +3740,22 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="S18" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -3734,38 +3776,26 @@
         </is>
       </c>
       <c r="AD18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE18" t="n">
         <v>1</v>
       </c>
       <c r="AF18" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG18" t="n">
         <v>1</v>
       </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>B. Mechele</t>
-        </is>
-      </c>
-      <c r="AI18" t="n">
-        <v>0.17586022</v>
-      </c>
-      <c r="AJ18" t="inlineStr">
-        <is>
-          <t>-0.08</t>
-        </is>
-      </c>
-      <c r="AK18" t="n">
-        <v>11</v>
-      </c>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
         <v>0</v>
       </c>
       <c r="AM18" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN18" t="n">
         <v>0</v>
@@ -3780,7 +3810,7 @@
         <v>0</v>
       </c>
       <c r="AR18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS18" t="n">
         <v>3</v>
@@ -3789,10 +3819,10 @@
         <v>0</v>
       </c>
       <c r="AU18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW18" t="n">
         <v>0</v>
@@ -3815,7 +3845,11 @@
       <c r="BC18" t="n">
         <v>0</v>
       </c>
-      <c r="BD18" t="inlineStr"/>
+      <c r="BD18" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
       <c r="BE18" t="n">
         <v>0</v>
       </c>
@@ -3823,7 +3857,7 @@
         <v>0</v>
       </c>
       <c r="BG18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -3839,17 +3873,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>L. Trossard</t>
+          <t>T. Meunier</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 10</t>
+          <t xml:space="preserve"> 15</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3859,12 +3893,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>8qwpdf5jof7o6yy47v6iv11hx</t>
+          <t>bb6glt8n0ar47cmhmj6gnfiz9</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -3881,35 +3915,25 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>56</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>LW</t>
-        </is>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="S19" t="n">
-        <v>45</v>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>LW</t>
-        </is>
-      </c>
-      <c r="U19" t="n">
-        <v>11</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
@@ -3927,68 +3951,68 @@
         </is>
       </c>
       <c r="AD19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE19" t="n">
         <v>1</v>
       </c>
       <c r="AF19" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG19" t="n">
         <v>1</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>L. Trossard</t>
+          <t>T. Meunier</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.39674971</v>
+        <v>0.76890101</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>+0.14</t>
+          <t>+0.37</t>
         </is>
       </c>
       <c r="AK19" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>95</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS19" t="n">
         <v>7</v>
       </c>
-      <c r="AL19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM19" t="n">
-        <v>56</v>
-      </c>
-      <c r="AN19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ19" t="n">
-        <v>4</v>
-      </c>
-      <c r="AR19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS19" t="n">
-        <v>0</v>
-      </c>
       <c r="AT19" t="n">
         <v>0</v>
       </c>
       <c r="AU19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AV19" t="n">
         <v>0</v>
       </c>
       <c r="AW19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX19" t="n">
         <v>0</v>
@@ -4008,19 +4032,15 @@
       <c r="BC19" t="n">
         <v>0</v>
       </c>
-      <c r="BD19" t="inlineStr">
-        <is>
-          <t>FWD</t>
-        </is>
-      </c>
+      <c r="BD19" t="inlineStr"/>
       <c r="BE19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BF19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BG19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -4036,17 +4056,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A. Onana</t>
+          <t>T. Castagne</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 24</t>
+          <t xml:space="preserve"> 21</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4056,12 +4076,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>do3duah478rhz9cg2icde4h9m</t>
+          <t>p87gxg8kc9ta6iipqt5fxmtx</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -4091,7 +4111,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="S20" t="n">
@@ -4122,26 +4142,26 @@
         <v>1</v>
       </c>
       <c r="AF20" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="AG20" t="n">
         <v>2</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>A. Onana</t>
+          <t>T. Castagne</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.33065845</v>
+        <v>0.23286301</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>+0.07</t>
+          <t>-0.17</t>
         </is>
       </c>
       <c r="AK20" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="AL20" t="n">
         <v>0</v>
@@ -4156,22 +4176,22 @@
         <v>0</v>
       </c>
       <c r="AP20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AS20" t="n">
         <v>1</v>
       </c>
       <c r="AT20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AV20" t="n">
         <v>1</v>
@@ -4180,7 +4200,7 @@
         <v>0</v>
       </c>
       <c r="AX20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY20" t="n">
         <v>0</v>
@@ -4202,7 +4222,7 @@
         <v>0</v>
       </c>
       <c r="BF20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG20" t="n">
         <v>0</v>
@@ -4221,17 +4241,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C. De Ketelaere</t>
+          <t>Y. Tielemans</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 17</t>
+          <t xml:space="preserve"> 8</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4241,12 +4261,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>7ox43isyywsnrfcd56nm65be</t>
+          <t>eo4uva2gnx08xdazfaqzyz2dx</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -4263,35 +4283,25 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>56</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>RW</t>
-        </is>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="S21" t="n">
-        <v>45</v>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>RW</t>
-        </is>
-      </c>
-      <c r="U21" t="n">
-        <v>11</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
@@ -4309,28 +4319,28 @@
         </is>
       </c>
       <c r="AD21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE21" t="n">
         <v>1</v>
       </c>
       <c r="AF21" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG21" t="n">
         <v>1</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>C. De Ketelaere</t>
+          <t>Y. Tielemans</t>
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>1.05464237</v>
+        <v>1.4175343</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>+0.80</t>
+          <t>+1.01</t>
         </is>
       </c>
       <c r="AK21" t="n">
@@ -4340,7 +4350,7 @@
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN21" t="n">
         <v>0</v>
@@ -4349,25 +4359,25 @@
         <v>0</v>
       </c>
       <c r="AP21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AQ21" t="n">
         <v>1</v>
       </c>
       <c r="AR21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AS21" t="n">
         <v>2</v>
       </c>
       <c r="AT21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AU21" t="n">
         <v>1</v>
       </c>
       <c r="AV21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW21" t="n">
         <v>0</v>
@@ -4390,15 +4400,19 @@
       <c r="BC21" t="n">
         <v>0</v>
       </c>
-      <c r="BD21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
       <c r="BE21" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="BF21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BG21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -4414,17 +4428,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>K. De Bruyne</t>
+          <t>N. Ngoy</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 7</t>
+          <t xml:space="preserve"> 25</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4434,12 +4448,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>c2jqa9vozhqu7x79h5rr2n1ed</t>
+          <t>a5jrqzijth7e3uxl4phi83sdm</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -4456,22 +4470,22 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="S22" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -4492,65 +4506,65 @@
         </is>
       </c>
       <c r="AD22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE22" t="n">
         <v>1</v>
       </c>
       <c r="AF22" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="AG22" t="n">
         <v>1</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>K. De Bruyne</t>
+          <t>N. Ngoy</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.45734978</v>
+        <v>0.39949639</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>+0.20</t>
+          <t>-0.00</t>
         </is>
       </c>
       <c r="AK22" t="n">
+        <v>11</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>95</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR22" t="n">
         <v>5</v>
       </c>
-      <c r="AL22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM22" t="n">
-        <v>56</v>
-      </c>
-      <c r="AN22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP22" t="n">
-        <v>2</v>
-      </c>
-      <c r="AQ22" t="n">
-        <v>2</v>
-      </c>
-      <c r="AR22" t="n">
-        <v>2</v>
-      </c>
       <c r="AS22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AT22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AU22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW22" t="n">
         <v>0</v>
@@ -4573,19 +4587,15 @@
       <c r="BC22" t="n">
         <v>0</v>
       </c>
-      <c r="BD22" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
+      <c r="BD22" t="inlineStr"/>
       <c r="BE22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BF22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BG22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -4601,17 +4611,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>J. Doku</t>
+          <t>B. Mechele</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 11</t>
+          <t xml:space="preserve"> 4</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4621,12 +4631,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>85gmjxvy1g5aj1lcizegwuaui</t>
+          <t>l6y4o9t2b0jxaxo85oztok45</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -4643,35 +4653,25 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>56</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S23" t="n">
-        <v>45</v>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="U23" t="n">
-        <v>11</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
@@ -4689,38 +4689,38 @@
         </is>
       </c>
       <c r="AD23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE23" t="n">
         <v>1</v>
       </c>
       <c r="AF23" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG23" t="n">
         <v>1</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>J. Doku</t>
+          <t>B. Mechele</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.10813124</v>
+        <v>1.05992592</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>+0.66</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN23" t="n">
         <v>0</v>
@@ -4729,28 +4729,28 @@
         <v>0</v>
       </c>
       <c r="AP23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS23" t="n">
         <v>5</v>
       </c>
-      <c r="AR23" t="n">
-        <v>5</v>
-      </c>
-      <c r="AS23" t="n">
-        <v>0</v>
-      </c>
       <c r="AT23" t="n">
         <v>1</v>
       </c>
       <c r="AU23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AV23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX23" t="n">
         <v>0</v>
@@ -4770,19 +4770,15 @@
       <c r="BC23" t="n">
         <v>0</v>
       </c>
-      <c r="BD23" t="inlineStr">
-        <is>
-          <t>FWD</t>
-        </is>
-      </c>
+      <c r="BD23" t="inlineStr"/>
       <c r="BE23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BF23" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="BG23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -4798,32 +4794,32 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>M. De Cuyper</t>
+          <t>L. Trossard</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 5</t>
+          <t xml:space="preserve"> 10</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>bjhjz96omjukrg6tj3mny39t6</t>
+          <t>8qwpdf5jof7o6yy47v6iv11hx</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -4832,37 +4828,43 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K24" t="n">
-        <v>55</v>
-      </c>
-      <c r="L24" t="n">
-        <v>2</v>
-      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="N24" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" t="inlineStr"/>
+        <v>95</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
       <c r="P24" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="S24" t="n">
-        <v>1</v>
-      </c>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
+        <v>45</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="U24" t="n">
+        <v>50</v>
+      </c>
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr"/>
@@ -4880,38 +4882,38 @@
         </is>
       </c>
       <c r="AD24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF24" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AG24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
-          <t>M. De Cuyper</t>
+          <t>L. Trossard</t>
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>0</v>
+        <v>1.08448248</v>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>-0.26</t>
+          <t>+0.68</t>
         </is>
       </c>
       <c r="AK24" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="AL24" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="AM24" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="AN24" t="n">
         <v>0</v>
@@ -4920,13 +4922,13 @@
         <v>0</v>
       </c>
       <c r="AP24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AQ24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AR24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS24" t="n">
         <v>0</v>
@@ -4935,7 +4937,7 @@
         <v>0</v>
       </c>
       <c r="AU24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AV24" t="n">
         <v>0</v>
@@ -4963,17 +4965,17 @@
       </c>
       <c r="BD24" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>FWD</t>
         </is>
       </c>
       <c r="BE24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BF24" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BG24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -4989,68 +4991,66 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>N. Raskin</t>
+          <t>A. Onana</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 23</t>
+          <t xml:space="preserve"> 24</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>do3duah478rhz9cg2icde4h9m</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>rmruexgp6l6ar57aq8xffg4q</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K25" t="n">
-        <v>56</v>
-      </c>
-      <c r="L25" t="n">
-        <v>2</v>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="N25" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="S25" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
@@ -5074,35 +5074,35 @@
         <v>0</v>
       </c>
       <c r="AE25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF25" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG25" t="n">
         <v>2</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>N. Raskin</t>
+          <t>A. Onana</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>0</v>
+        <v>0.32994343</v>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>-0.26</t>
+          <t>-0.07</t>
         </is>
       </c>
       <c r="AK25" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="AL25" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="AM25" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AN25" t="n">
         <v>0</v>
@@ -5117,19 +5117,19 @@
         <v>0</v>
       </c>
       <c r="AR25" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AS25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU25" t="n">
         <v>0</v>
       </c>
       <c r="AV25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW25" t="n">
         <v>0</v>
@@ -5160,6 +5160,1552 @@
         <v>0</v>
       </c>
       <c r="BG25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>aw4mhrfav7b5r7d4lc6dwz1g4</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>C. De Ketelaere</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 17</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>7ox43isyywsnrfcd56nm65be</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>65</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>65</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>45</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="U26" t="n">
+        <v>20</v>
+      </c>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="AD26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>C. De Ketelaere</t>
+        </is>
+      </c>
+      <c r="AI26" t="n">
+        <v>1.30025654</v>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>+0.90</t>
+        </is>
+      </c>
+      <c r="AK26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>65</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>aw4mhrfav7b5r7d4lc6dwz1g4</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>K. De Bruyne</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 7</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>c2jqa9vozhqu7x79h5rr2n1ed</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>85</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>85</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>85</v>
+      </c>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="AD27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>K. De Bruyne</t>
+        </is>
+      </c>
+      <c r="AI27" t="n">
+        <v>0.7895290100000001</v>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>+0.39</t>
+        </is>
+      </c>
+      <c r="AK27" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>85</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD27" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="BE27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF27" t="n">
+        <v>6</v>
+      </c>
+      <c r="BG27" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>aw4mhrfav7b5r7d4lc6dwz1g4</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>J. Doku</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>85gmjxvy1g5aj1lcizegwuaui</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>85</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>85</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="S28" t="n">
+        <v>45</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="U28" t="n">
+        <v>40</v>
+      </c>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="AD28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>J. Doku</t>
+        </is>
+      </c>
+      <c r="AI28" t="n">
+        <v>0.2221491499999999</v>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>-0.18</t>
+        </is>
+      </c>
+      <c r="AK28" t="n">
+        <v>16</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>85</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>8</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD28" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
+      <c r="BE28" t="n">
+        <v>7</v>
+      </c>
+      <c r="BF28" t="n">
+        <v>9</v>
+      </c>
+      <c r="BG28" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>aw4mhrfav7b5r7d4lc6dwz1g4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>M. De Cuyper</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 5</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>bjhjz96omjukrg6tj3mny39t6</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>55</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>40</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>55</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>95</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="S29" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="U29" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="AD29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>M. De Cuyper</t>
+        </is>
+      </c>
+      <c r="AI29" t="n">
+        <v>0.1033109</v>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>-0.30</t>
+        </is>
+      </c>
+      <c r="AK29" t="n">
+        <v>20</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>55</v>
+      </c>
+      <c r="AM29" t="n">
+        <v>95</v>
+      </c>
+      <c r="AN29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR29" t="n">
+        <v>4</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD29" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="BE29" t="n">
+        <v>4</v>
+      </c>
+      <c r="BF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>aw4mhrfav7b5r7d4lc6dwz1g4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>R. Lukaku</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 9</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>8qgbxff7xlg0zjtyees7ljljp</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>65</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
+        <v>30</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="n">
+        <v>65</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>95</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S30" t="n">
+        <v>30</v>
+      </c>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="AD30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>R. Lukaku</t>
+        </is>
+      </c>
+      <c r="AI30" t="n">
+        <v>0.08050533000000004</v>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>-0.32</t>
+        </is>
+      </c>
+      <c r="AK30" t="n">
+        <v>22</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>65</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>95</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD30" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
+      <c r="BE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>aw4mhrfav7b5r7d4lc6dwz1g4</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>H. Vanaken</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 20</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>x3g0yyxs0j4o8fxphxtf0st1</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>85</v>
+      </c>
+      <c r="L31" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>10</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="n">
+        <v>85</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>95</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="S31" t="n">
+        <v>10</v>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="AD31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>H. Vanaken</t>
+        </is>
+      </c>
+      <c r="AI31" t="n">
+        <v>0.01892452999999999</v>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>-0.38</t>
+        </is>
+      </c>
+      <c r="AK31" t="n">
+        <v>26</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>85</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>95</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD31" t="inlineStr"/>
+      <c r="BE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>aw4mhrfav7b5r7d4lc6dwz1g4</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>N. Raskin</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 23</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>rmruexgp6l6ar57aq8xffg4q</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>55</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>40</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>55</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>95</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="U32" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="AD32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>N. Raskin</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>0.23629699</v>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>-0.17</t>
+        </is>
+      </c>
+      <c r="AK32" t="n">
+        <v>14</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>55</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>95</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD32" t="inlineStr"/>
+      <c r="BE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>aw4mhrfav7b5r7d4lc6dwz1g4</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>M. Fernandez-Pardo</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2branork7cntloew47tif7das</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>85</v>
+      </c>
+      <c r="L33" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>10</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="n">
+        <v>85</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>95</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>10</v>
+      </c>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>pfvmhackqyhhk02majd2tb8l</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="AD33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>M. Fernandez-Pardo</t>
+        </is>
+      </c>
+      <c r="AI33" t="n">
+        <v>0.05194948000000001</v>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>-0.35</t>
+        </is>
+      </c>
+      <c r="AK33" t="n">
+        <v>24</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>85</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>95</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD33" t="inlineStr"/>
+      <c r="BE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG33" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>